<commit_message>
stock mode w news feature using claude
</commit_message>
<xml_diff>
--- a/etf_comparison.xlsx
+++ b/etf_comparison.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ETFS Analyzed: SPY, QQQ, VTI, ARKK</t>
+          <t>ETFS Analyzed: VOO, QQQ, ARKK, VTI, SPY</t>
         </is>
       </c>
     </row>
@@ -533,98 +533,119 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SPY: NVIDIA Corp (7.3%)</t>
+          <t>VOO: NVIDIA Corp (7.3%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>QQQ: NVIDIA Corp (8.4%)</t>
+          <t>QQQ: NVIDIA Corp (8.7%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VTI: NVIDIA Corp (6.2%)</t>
+          <t>ARKK: Tesla Inc (10.4%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ARKK: Tesla Inc (10.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+          <t>VTI: NVIDIA Corp (6.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SPY: NVIDIA Corp (7.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Larget Sector per ETF</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SPY: Technology (33.08%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>QQQ: Technology (50.0%)</t>
+          <t>VOO: Technology (33.14%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VTI: Technology (31.11%)</t>
+          <t>QQQ: Technology (50.54%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ARKK: Healthcare (30.19%)</t>
+          <t>ARKK: Healthcare (29.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VTI: Technology (31.11%)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SPY: Technology (33.56%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Overlap Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ARKK vs ARKK: 1 stocks in common - 1.9% of SPY, 10.4% of ARKK</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ARKK vs ARKK: 1 stocks in common - 3.9% of QQQ, 10.4% of ARKK</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ARKK vs ARKK: 1 stocks in common - 1.7% of VTI, 10.4% of ARKK</t>
+          <t>SPY vs SPY: 10 stocks in common - 36.3% of VOO, 36.4% of SPY</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ARKK vs ARKK: 10 stocks in common - 51.3% of ARKK, 51.3% of ARKK</t>
+          <t>SPY vs SPY: 9 stocks in common - 43.4% of QQQ, 34.8% of SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SPY vs SPY: 1 stocks in common - 10.4% of ARKK, 1.9% of SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SPY vs SPY: 10 stocks in common - 31.9% of VTI, 36.4% of SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SPY vs SPY: 10 stocks in common - 36.4% of SPY, 36.4% of SPY</t>
         </is>
       </c>
     </row>
@@ -639,11 +660,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
@@ -682,11 +703,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.07315240000000001</v>
+        <v>0.0730978</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -702,11 +723,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.06632059999999999</v>
+        <v>0.066271804</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -722,11 +743,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.049592</v>
+        <v>0.0495553</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -742,11 +763,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0347069</v>
+        <v>0.0346825</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -762,11 +783,11 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0308148</v>
+        <v>0.0307936</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -782,11 +803,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.025636699</v>
+        <v>0.0256188</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -802,11 +823,11 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0246022</v>
+        <v>0.024585</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -822,11 +843,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.023982301</v>
+        <v>0.0239659</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -842,11 +863,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0192143</v>
+        <v>0.019201301</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -862,11 +883,11 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.015729701</v>
+        <v>0.0157195</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VOO</t>
         </is>
       </c>
     </row>
@@ -882,7 +903,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.08399419499999999</v>
+        <v>0.08671230000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -902,7 +923,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.0761501</v>
+        <v>0.0762364</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -922,7 +943,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0569425</v>
+        <v>0.056242198</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -942,7 +963,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.043793503</v>
+        <v>0.045746103</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -962,7 +983,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.0391901</v>
+        <v>0.037964202</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -982,7 +1003,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.0371346</v>
+        <v>0.0345264</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -993,16 +1014,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alphabet Inc Class A</t>
+          <t>Walmart Inc</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.0353833</v>
+        <v>0.034309197</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1013,16 +1034,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Walmart Inc</t>
+          <t>Alphabet Inc Class A</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0336763</v>
+        <v>0.0342554</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1042,7 +1063,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.032848798</v>
+        <v>0.031918097</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1062,7 +1083,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.0294376</v>
+        <v>0.030026</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1073,400 +1094,600 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NVIDIA Corp</t>
+          <t>Tesla Inc</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.0617275</v>
+        <v>0.1040665</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Apple Inc</t>
+          <t>CRISPR Therapeutics AG</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.058908</v>
+        <v>0.0621205</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Microsoft Corp</t>
+          <t>Tempus AI Inc Class A common stock</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.044049602</v>
+        <v>0.048905402</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Amazon.com Inc</t>
+          <t>Shopify Inc Registered Shs -A- Subord Vtg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.030490201</v>
+        <v>0.0479929</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alphabet Inc Class A</t>
+          <t>Circle Internet Group Inc Ordinary Shares - Class A</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.0273606</v>
+        <v>0.045194604</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>COIN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Broadcom Inc</t>
+          <t>Coinbase Global Inc Ordinary Shares - Class A</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.0227725</v>
+        <v>0.044088896</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alphabet Inc Class C</t>
+          <t>Robinhood Markets Inc Class A</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.021610899</v>
+        <v>0.042701602</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Meta Platforms Inc Class A</t>
+          <t>Roku Inc Class A</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.021303201</v>
+        <v>0.039868</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tesla Inc</t>
+          <t>Advanced Micro Devices Inc</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.0171717</v>
+        <v>0.039659098</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Berkshire Hathaway Inc Class B</t>
+          <t>Palantir Technologies Inc Ordinary Shares - Class A</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.013682701</v>
+        <v>0.0357451</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>ARKK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tesla Inc</t>
+          <t>NVIDIA Corp</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.1043495</v>
+        <v>0.0617275</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CRSP</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CRISPR Therapeutics AG</t>
+          <t>Apple Inc</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.06925969999999999</v>
+        <v>0.058908</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tempus AI Inc Class A common stock</t>
+          <t>Microsoft Corp</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.0522995</v>
+        <v>0.044049602</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Roku Inc Class A</t>
+          <t>Amazon.com Inc</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.0504594</v>
+        <v>0.030490201</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Shopify Inc Registered Shs -A- Subord Vtg</t>
+          <t>Alphabet Inc Class A</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.0441159</v>
+        <v>0.0273606</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>COIN</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Coinbase Global Inc Ordinary Shares - Class A</t>
+          <t>Broadcom Inc</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.0406488</v>
+        <v>0.0227725</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Robinhood Markets Inc Class A</t>
+          <t>Alphabet Inc Class C</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.039859198</v>
+        <v>0.021610899</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BEAM</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Beam Therapeutics Inc</t>
+          <t>Meta Platforms Inc Class A</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.0376935</v>
+        <v>0.021303201</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices Inc</t>
+          <t>Tesla Inc</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.0374948</v>
+        <v>0.0171717</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RBLX</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Roblox Corp Ordinary Shares - Class A</t>
+          <t>Berkshire Hathaway Inc Class B</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.0371127</v>
+        <v>0.013682701</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>VTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NVIDIA Corp</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0.07559059999999999</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Apple Inc</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0.066458</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Microsoft Corp</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0.049028</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Amazon.com Inc</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0.0362905</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Alphabet Inc Class A</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>0.0298607</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Broadcom Inc</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0.0261756</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Alphabet Inc Class C</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>0.023929501</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Meta Platforms Inc Class A</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>0.0223206</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tesla Inc</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>0.0186473</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BRK-B</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Berkshire Hathaway Inc Class B</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>0.015672099</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>SPY</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1489,8 +1710,9 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="64" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1506,34 +1728,39 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Overlap Weight in VOO</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Overlap Weight in QQQ</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Shared Tickers</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Overlap Weight in ARKK</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Overlap Weight in VTI</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
           <t>Overlap Weight in SPY</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Overlap Weight in QQQ</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Shared Tickers</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Overlap Weight in VTI</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Overlap Weight in ARKK</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SPY vs QQQ</t>
+          <t>VOO vs QQQ</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1546,7 +1773,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>43.4%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1556,87 +1783,91 @@
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SPY vs VTI</t>
+          <t>VOO vs ARKK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>36.4%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AAPL, AMZN, AVGO, BRK-B, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>31.9%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPY vs ARKK</t>
+          <t>VOO vs VTI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>36.3%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>AAPL, AMZN, AVGO, BRK-B, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10.4%</t>
-        </is>
-      </c>
+          <t>31.9%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>QQQ vs VTI</t>
+          <t>VOO vs SPY</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>43.5%</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>36.3%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AAPL, AMZN, AVGO, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>30.5%</t>
-        </is>
-      </c>
+          <t>AAPL, AMZN, AVGO, BRK-B, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>36.4%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1650,7 +1881,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1658,37 +1889,151 @@
           <t>TSLA</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>10.4%</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VTI vs ARKK</t>
+          <t>QQQ vs VTI</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>43.4%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AAPL, AMZN, AVGO, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>30.5%</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QQQ vs SPY</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>43.4%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AAPL, AMZN, AVGO, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>34.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ARKK vs VTI</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>TSLA</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>1.7%</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ARKK vs SPY</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>10.4%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VTI vs SPY</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AAPL, AMZN, AVGO, BRK-B, GOOG, GOOGL, META, MSFT, NVDA, TSLA</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>31.9%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>36.4%</t>
         </is>
       </c>
     </row>
@@ -1703,7 +2048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1711,6 +2056,7 @@
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1721,22 +2067,27 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>ARKK</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>VTI</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>SPY</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>VTI</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>ARKK</t>
         </is>
       </c>
     </row>
@@ -1753,10 +2104,13 @@
         <v>0.1</v>
       </c>
       <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
         <v>2.5</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
+      <c r="F2" t="n">
+        <v>1.95</v>
       </c>
     </row>
     <row r="3">
@@ -1766,16 +2120,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.11</v>
+        <v>10.13</v>
       </c>
       <c r="C3" t="n">
-        <v>12.51</v>
+        <v>12.62</v>
       </c>
       <c r="D3" t="n">
+        <v>13.89</v>
+      </c>
+      <c r="E3" t="n">
         <v>10.08</v>
       </c>
-      <c r="E3" t="n">
-        <v>12.93</v>
+      <c r="F3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1785,16 +2142,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.93</v>
+        <v>1.94</v>
       </c>
       <c r="C4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>2.19</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
+      <c r="F4" t="n">
+        <v>1.9</v>
       </c>
     </row>
     <row r="5">
@@ -1804,16 +2164,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.43</v>
+        <v>5.44</v>
       </c>
       <c r="C5" t="n">
-        <v>8.59</v>
+        <v>8.58</v>
       </c>
       <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>5.13</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
+      <c r="F5" t="n">
+        <v>5.25</v>
       </c>
     </row>
     <row r="6">
@@ -1823,16 +2186,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33.08</v>
+        <v>33.14</v>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>50.54</v>
       </c>
       <c r="D6" t="n">
+        <v>25.28</v>
+      </c>
+      <c r="E6" t="n">
         <v>31.11</v>
       </c>
-      <c r="E6" t="n">
-        <v>24.56</v>
+      <c r="F6" t="n">
+        <v>33.56</v>
       </c>
     </row>
     <row r="7">
@@ -1842,16 +2208,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10.73</v>
+        <v>10.75</v>
       </c>
       <c r="C7" t="n">
-        <v>16.44</v>
+        <v>16.06</v>
       </c>
       <c r="D7" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E7" t="n">
         <v>9.880000000000001</v>
       </c>
-      <c r="E7" t="n">
-        <v>12.06</v>
+      <c r="F7" t="n">
+        <v>10.48</v>
       </c>
     </row>
     <row r="8">
@@ -1861,16 +2230,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12.26</v>
+        <v>12.1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="D8" t="n">
+        <v>16.42</v>
+      </c>
+      <c r="E8" t="n">
         <v>12.37</v>
       </c>
-      <c r="E8" t="n">
-        <v>14.15</v>
+      <c r="F8" t="n">
+        <v>12.35</v>
       </c>
     </row>
     <row r="9">
@@ -1883,13 +2255,16 @@
         <v>2.49</v>
       </c>
       <c r="C9" t="n">
-        <v>1.57</v>
+        <v>1.54</v>
       </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>2.45</v>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
+      <c r="F9" t="n">
+        <v>2.54</v>
       </c>
     </row>
     <row r="10">
@@ -1899,16 +2274,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8.66</v>
+        <v>8.68</v>
       </c>
       <c r="C10" t="n">
-        <v>3.39</v>
+        <v>3.26</v>
       </c>
       <c r="D10" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="E10" t="n">
         <v>10.23</v>
       </c>
-      <c r="E10" t="n">
-        <v>6.1</v>
+      <c r="F10" t="n">
+        <v>8.470000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1918,16 +2296,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.48</v>
+        <v>3.49</v>
       </c>
       <c r="C11" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>3.64</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
+      <c r="F11" t="n">
+        <v>4.02</v>
       </c>
     </row>
     <row r="12">
@@ -1937,16 +2318,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.84</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>5.26</v>
+        <v>5.11</v>
       </c>
       <c r="D12" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="E12" t="n">
         <v>10.43</v>
       </c>
-      <c r="E12" t="n">
-        <v>30.19</v>
+      <c r="F12" t="n">
+        <v>9.470000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>